<commit_message>
docs: remove background color fills from docs/test_cases.xlsx
</commit_message>
<xml_diff>
--- a/docs/test_cases.xlsx
+++ b/docs/test_cases.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,6 +35,17 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -92,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -110,6 +121,15 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -494,987 +514,987 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Module</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Objective</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Input Data</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Steps</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>Technique</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>TC-MOD-01</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>models</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="9" t="inlineStr">
         <is>
           <t>validate_expense</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="9" t="inlineStr">
         <is>
           <t>Accept a fully valid expense entry</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t>expense_tracker.models imported; all categories available</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="9" t="inlineStr">
         <is>
           <t>amount=45.50, desc=Groceries, category=Food, date=2026-10-15</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="9" t="inlineStr">
         <is>
           <t>1. Call validate_expense with valid inputs
 2. Inspect returned dict</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="9" t="inlineStr">
         <is>
           <t>Returns dict with no errors key; amount == Decimal(45.50)</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" s="9" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="8" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="8" t="inlineStr">
         <is>
           <t>ECP – Valid partition</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>TC-MOD-02</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>models</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>validate_expense</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>Reject blank description</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>expense_tracker.models imported</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>amount=10.00, description=   , category=Food, date=2026-10-15</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>1. Call validate_expense with whitespace-only description
 2. Inspect errors dict</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>errors[description] == Description is required.</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr">
+      <c r="I3" s="9" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="K3" s="8" t="inlineStr">
         <is>
           <t>ECP – Invalid partition (missing description)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>TC-MOD-03</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>models</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>validate_expense</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Reject negative amount</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>expense_tracker.models imported</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>amount=-1.00, desc=Refund, category=Bills, date=2026-10-15</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="9" t="inlineStr">
         <is>
           <t>1. Call validate_expense with negative amount
 2. Inspect errors dict</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="9" t="inlineStr">
         <is>
           <t>errors[amount] == Amount must be greater than \.</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="9" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J4" s="8" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K4" s="8" t="inlineStr">
         <is>
           <t>BVA – Below lower boundary (0)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>TC-MOD-04</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>models</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>validate_expense</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Reject amount exceeding maximum</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>expense_tracker.models imported; MAX_AMOUNT = 1000000</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>amount=1000000.01, desc=Yacht, category=Shopping, date=2026-10-15</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>1. Call validate_expense with amount &gt; 1000000
 2. Inspect errors dict</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>errors[amount] == That amount looks too large.</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="I5" s="9" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" s="8" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
         <is>
           <t>BVA – Above upper boundary (1000000)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>TC-MOD-05</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>models</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>validate_expense</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Reject invalid category</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>expense_tracker.models imported; valid categories in CATEGORIES constant</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>amount=20.00, desc=Movie, category=Entertainment, date=2026-10-15</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>1. Call validate_expense with unknown category
 2. Inspect errors dict</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>errors[category] == Choose a valid category.</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" s="9" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" s="8" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K6" s="8" t="inlineStr">
         <is>
           <t>ECP – Invalid partition (unknown category)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>TC-MOD-06</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>models</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>validate_expense</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>Accept minimum valid amount (boundary)</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>expense_tracker.models imported</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>amount=0.01, desc=Penny candy, category=Other, date=2026-10-15</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>1. Call validate_expense with amount=0.01
 2. Confirm no errors returned</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>Returns dict with no errors key; amount == Decimal(0.01)</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="I7" s="9" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="J7" s="8" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="K7" s="8" t="inlineStr">
         <is>
           <t>BVA – Exact lower boundary (0.01)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>TC-FMT-01</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>formatting</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>format_currency</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Format positive amount with 2 decimal places</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>expense_tracker.formatting imported</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>amount=Decimal(1234.56)</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>1. Call format_currency(Decimal(1234.56))
 2. Compare returned string</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" s="9" t="inlineStr">
         <is>
           <t>Returns \,234.56</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="I8" s="9" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J8" s="8" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K8" s="8" t="inlineStr">
         <is>
           <t>ECP – Valid positive amount</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>TC-FMT-02</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>formatting</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>format_currency</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Format zero amount</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>expense_tracker.formatting imported</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>amount=Decimal(0)</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr">
         <is>
           <t>1. Call format_currency(Decimal(0))
 2. Compare returned string</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="9" t="inlineStr">
         <is>
           <t>Returns \.00</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="I9" s="9" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="J9" s="8" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="K9" s="8" t="inlineStr">
         <is>
           <t>BVA – Zero boundary</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>TC-FMT-03</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>formatting</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>format_date</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Format a date object to readable string</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>expense_tracker.formatting imported</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>date=date(2026, 10, 15)</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="9" t="inlineStr">
         <is>
           <t>1. Call format_date(date(2026, 10, 15))
 2. Compare returned string</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H10" s="9" t="inlineStr">
         <is>
           <t>Returns Oct 15, 2026</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="I10" s="9" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="J10" s="8" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K10" s="8" t="inlineStr">
         <is>
           <t>ECP – Valid date object</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>TC-STA-01</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>stats</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>total_of</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>Sum amounts for a single-item list</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>expense_tracker.stats imported; Expense available</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>expenses=[Expense(amount=Decimal(50.00), ...)]</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
         <is>
           <t>1. Call total_of(expenses)
 2. Assert return value</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H11" s="9" t="inlineStr">
         <is>
           <t>Returns Decimal(50.00)</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="I11" s="9" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="J11" s="8" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr">
+      <c r="K11" s="8" t="inlineStr">
         <is>
           <t>ECP – Single-element list</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>TC-STA-02</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>stats</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>total_of</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>Return zero for empty list</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>expense_tracker.stats imported</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>expenses=[]</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" s="9" t="inlineStr">
         <is>
           <t>1. Call total_of([])
 2. Assert return value</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H12" s="9" t="inlineStr">
         <is>
           <t>Returns Decimal(0) or 0</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="I12" s="9" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J12" s="8" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K12" s="8" t="inlineStr">
         <is>
           <t>ECP – Empty list boundary</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>TC-STA-03</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>stats</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>expenses_in_month</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>Filter expenses to matching month and year</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>expense_tracker.stats imported; Expense objects with dates</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>expenses=[exp(2026-10-05), exp(2026-09-20)], year=2026, month=10</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
         <is>
           <t>1. Call expenses_in_month(expenses, 2026, 10)
 2. Check returned list</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="H13" s="9" t="inlineStr">
         <is>
           <t>Returns only October 2026 expense; September expense excluded</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="I13" s="9" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="J13" s="8" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="K13" s="8" t="inlineStr">
         <is>
           <t>ECP – Filtering by month/year</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>TC-STA-04</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>stats</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>category_breakdown</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>Produce correct percentage breakdown for two categories</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>expense_tracker.stats imported; expenses with two distinct categories</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>expenses=[exp(Food,60), exp(Bills,40)], total=100</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G14" s="9" t="inlineStr">
         <is>
           <t>1. Call category_breakdown(expenses)
 2. Inspect returned list</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="H14" s="9" t="inlineStr">
         <is>
           <t>Food -&gt; 60%, Bills -&gt; 40%; percentages sum to 100%</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="I14" s="9" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="J14" s="8" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K14" s="8" t="inlineStr">
         <is>
           <t>ECP – Multi-category breakdown</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>TC-STA-05</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>stats</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>monthly_trend</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>Aggregate expenses across multiple months</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E15" s="9" t="inlineStr">
         <is>
           <t>expense_tracker.stats imported; expenses spanning three months</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>expenses=[exp(2026-08), exp(2026-09), exp(2026-10)]</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="G15" s="9" t="inlineStr">
         <is>
           <t>1. Call monthly_trend(expenses)
 2. Verify 3 entries with correct totals</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H15" s="9" t="inlineStr">
         <is>
           <t>Returns 3 trend points, one per month, with correct summed totals</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="I15" s="9" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="J15" s="8" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="K15" s="8" t="inlineStr">
         <is>
           <t>ECP – Multi-month aggregation</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>TC-CSV-01</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>models</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>validate_expense</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>CSV-driven: valid standard expense (test_cases.csv row 1)</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t>tests/data/test_cases.csv present; pytest parametrize configured</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>amount=45.50, desc=Grocery shopping, category=Food, date=2026-10-15</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G16" s="9" t="inlineStr">
         <is>
           <t>1. pytest reads CSV row TC-CSV-01
 2. Calls validate_expense
 3. Asserts no errors</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="H16" s="9" t="inlineStr">
         <is>
           <t>Validation passes; amount Decimal == 45.50</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="I16" s="9" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="J16" s="8" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K16" s="8" t="inlineStr">
         <is>
           <t>Data-Driven – CSV row TC-CSV-01</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>TC-CSV-06</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>models</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>validate_expense</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>CSV-driven: amount exceeds maximum boundary (test_cases.csv row 6)</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E17" s="9" t="inlineStr">
         <is>
           <t>tests/data/test_cases.csv present; pytest parametrize configured</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>amount=1000000.01, desc=Luxury Yacht, category=Shopping, date=2026-10-15</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="G17" s="9" t="inlineStr">
         <is>
           <t>1. pytest reads CSV row TC-CSV-06
 2. Calls validate_expense
 3. Checks error field</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="H17" s="9" t="inlineStr">
         <is>
           <t>errors[amount] == That amount looks too large.</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr">
+      <c r="I17" s="9" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="J17" s="8" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="K17" s="5" t="inlineStr">
+      <c r="K17" s="8" t="inlineStr">
         <is>
           <t>Data-Driven – CSV row TC-CSV-06 / BVA</t>
         </is>

</xml_diff>